<commit_message>
feat(lakeshore): upgrade pack with technical architecture SVGs + enriched docs
</commit_message>
<xml_diff>
--- a/docs/build/lakeshore-enterprise-context/data_dictionary.xlsx
+++ b/docs/build/lakeshore-enterprise-context/data_dictionary.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E129"/>
+  <dimension ref="A1:E135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>5851</v>
+        <v>5852</v>
       </c>
     </row>
     <row r="9">
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>6058</v>
+        <v>6059</v>
       </c>
     </row>
     <row r="17">
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>6247</v>
+        <v>6248</v>
       </c>
     </row>
     <row r="18">
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>5976</v>
+        <v>5977</v>
       </c>
     </row>
     <row r="23">
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>6535</v>
+        <v>6536</v>
       </c>
     </row>
     <row r="31">
@@ -1422,32 +1422,32 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>source/03_strategy_initiatives/roadmap_2026_2027.svg</t>
+          <t>source/04_finance_performance/pnl_baseline.xlsx</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>svg</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>strategy_initiatives</t>
+          <t>finance_performance</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Corporate Strategy</t>
+          <t>Oracle Hyperion</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>2959</v>
+        <v>6528</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>source/04_finance_performance/pnl_baseline.xlsx</t>
+          <t>source/04_finance_performance/cash_working_capital.xlsx</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1462,22 +1462,22 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Oracle Hyperion</t>
+          <t>Kyriba TMS</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>6529</v>
+        <v>5797</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>source/04_finance_performance/cash_working_capital.xlsx</t>
+          <t>source/04_finance_performance/fpa_process.docx</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1487,17 +1487,17 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Kyriba TMS</t>
+          <t>OneStream</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>5812</v>
+        <v>38310</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>source/04_finance_performance/fpa_process.docx</t>
+          <t>source/04_finance_performance/forecasting_process.docx</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1516,13 +1516,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>38310</v>
+        <v>38306</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>source/04_finance_performance/forecasting_process.docx</t>
+          <t>source/04_finance_performance/close_process.docx</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1541,18 +1541,18 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>38306</v>
+        <v>38314</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>source/04_finance_performance/close_process.docx</t>
+          <t>source/04_finance_performance/management_reporting.pdf</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1562,22 +1562,22 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>OneStream</t>
+          <t>Power BI</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>38314</v>
+        <v>2819</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>source/04_finance_performance/management_reporting.pdf</t>
+          <t>source/04_finance_performance/kpi_catalog.xlsx</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1591,13 +1591,13 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>2819</v>
+        <v>6009</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>source/04_finance_performance/kpi_catalog.xlsx</t>
+          <t>source/04_finance_performance/value_pools.xlsx</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1612,22 +1612,22 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Power BI</t>
+          <t>FP&amp;A</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>6010</v>
+        <v>5775</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>source/04_finance_performance/value_pools.xlsx</t>
+          <t>source/04_finance_performance/monthly_management_pack.pdf</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1637,22 +1637,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>FP&amp;A</t>
+          <t>Power BI</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>5771</v>
+        <v>2730</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>source/04_finance_performance/monthly_management_pack.pdf</t>
+          <t>source/04_finance_performance/finance_calendar.csv</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>csv</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1662,22 +1662,22 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Power BI</t>
+          <t>OneStream</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>2730</v>
+        <v>525</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>source/04_finance_performance/finance_calendar.csv</t>
+          <t>source/04_finance_performance/working_capital_drivers.xlsx</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1687,17 +1687,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>OneStream</t>
+          <t>Kyriba TMS</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>535</v>
+        <v>5621</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>source/04_finance_performance/working_capital_drivers.xlsx</t>
+          <t>source/05_treasury_kyriba/kyriba_rollout_plan.xlsx</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>finance_performance</t>
+          <t>treasury_kyriba</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1716,13 +1716,13 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>5628</v>
+        <v>5673</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/kyriba_rollout_plan.xlsx</t>
+          <t>source/05_treasury_kyriba/bank_connectivity_inventory.xlsx</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1741,18 +1741,18 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>5684</v>
+        <v>5896</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/bank_connectivity_inventory.xlsx</t>
+          <t>source/05_treasury_kyriba/payment_process.docx</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1766,13 +1766,13 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>5891</v>
+        <v>38953</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/payment_process.docx</t>
+          <t>source/05_treasury_kyriba/kyriba_integration_design.docx</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1787,17 +1787,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Kyriba TMS</t>
+          <t>SAP S/4HANA</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>38221</v>
+        <v>38880</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/kyriba_integration_design.docx</t>
+          <t>source/05_treasury_kyriba/treasury_policy.docx</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1812,22 +1812,22 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>SAP S/4HANA</t>
+          <t>Treasury</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>38237</v>
+        <v>38366</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/treasury_policy.docx</t>
+          <t>source/05_treasury_kyriba/cash_positioning.xlsx</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1837,17 +1837,17 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Treasury</t>
+          <t>Kyriba TMS</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>38210</v>
+        <v>5774</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/cash_positioning.xlsx</t>
+          <t>source/05_treasury_kyriba/liquidity_forecasting.xlsx</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1866,13 +1866,13 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>5782</v>
+        <v>5823</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/liquidity_forecasting.xlsx</t>
+          <t>source/05_treasury_kyriba/debt_fx_exposure.xlsx</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1891,13 +1891,13 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>5827</v>
+        <v>5604</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/debt_fx_exposure.xlsx</t>
+          <t>source/05_treasury_kyriba/bank_fee_baseline.xlsx</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1916,18 +1916,18 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>5607</v>
+        <v>5764</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/bank_fee_baseline.xlsx</t>
+          <t>source/05_treasury_kyriba/treasury_controls.pdf</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1941,13 +1941,13 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>5770</v>
+        <v>2720</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/treasury_controls.pdf</t>
+          <t>source/05_treasury_kyriba/treasury_target_operating_model.pdf</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1966,18 +1966,18 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>2720</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/treasury_target_operating_model.pdf</t>
+          <t>source/05_treasury_kyriba/kyriba_rollout_risks_defects.xlsx</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1991,18 +1991,18 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>2460</v>
+        <v>6176</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/kyriba_rollout_risks_defects.xlsx</t>
+          <t>source/05_treasury_kyriba/kyriba_test_defects.csv</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>csv</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2016,43 +2016,43 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>6170</v>
+        <v>3743</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>source/05_treasury_kyriba/kyriba_test_defects.csv</t>
+          <t>source/06_it_systems_architecture/application_inventory.xlsx</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>treasury_kyriba</t>
+          <t>it_systems_architecture</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Kyriba TMS</t>
+          <t>ServiceNow CMDB</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>3708</v>
+        <v>10943</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>source/06_it_systems_architecture/application_inventory.xlsx</t>
+          <t>source/06_it_systems_architecture/erp_landscape.pdf</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2062,22 +2062,22 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ServiceNow CMDB</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>10953</v>
+        <v>4194</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>source/06_it_systems_architecture/erp_landscape.pdf</t>
+          <t>source/06_it_systems_architecture/hris_workday.docx</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2087,17 +2087,17 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Workday HCM</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>2712</v>
+        <v>38260</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>source/06_it_systems_architecture/hris_workday.docx</t>
+          <t>source/06_it_systems_architecture/procurement_systems.docx</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2112,17 +2112,17 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Workday HCM</t>
+          <t>Coupa</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>38232</v>
+        <v>38262</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>source/06_it_systems_architecture/procurement_systems.docx</t>
+          <t>source/06_it_systems_architecture/identity_sso.docx</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2137,17 +2137,17 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Coupa</t>
+          <t>Azure Active Directory</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>38231</v>
+        <v>38276</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>source/06_it_systems_architecture/identity_sso.docx</t>
+          <t>source/06_it_systems_architecture/data_platforms.docx</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2162,22 +2162,22 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Azure Active Directory</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>38243</v>
+        <v>38767</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>source/06_it_systems_architecture/data_platforms.docx</t>
+          <t>source/06_it_systems_architecture/finance_systems.xlsx</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2187,17 +2187,17 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Snowflake</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>38226</v>
+        <v>5615</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>source/06_it_systems_architecture/finance_systems.xlsx</t>
+          <t>source/06_it_systems_architecture/reporting_tools.xlsx</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2212,17 +2212,17 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Power BI</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>5614</v>
+        <v>5560</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>source/06_it_systems_architecture/reporting_tools.xlsx</t>
+          <t>source/06_it_systems_architecture/security_tools.xlsx</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2237,17 +2237,17 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Power BI</t>
+          <t>Sentinel</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>5560</v>
+        <v>5574</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>source/06_it_systems_architecture/security_tools.xlsx</t>
+          <t>source/06_it_systems_architecture/legacy_applications.xlsx</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2262,22 +2262,22 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Sentinel</t>
+          <t>ServiceNow CMDB</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>5573</v>
+        <v>6099</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>source/06_it_systems_architecture/legacy_applications.xlsx</t>
+          <t>source/06_it_systems_architecture/integration_architecture.pdf</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2287,22 +2287,22 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ServiceNow CMDB</t>
+          <t>SAP PI/PO</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>6088</v>
+        <v>4107</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>source/06_it_systems_architecture/integration_architecture.pdf</t>
+          <t>source/06_it_systems_architecture/interface_inventory.xlsx</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2316,38 +2316,38 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>2442</v>
+        <v>8445</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>source/06_it_systems_architecture/current_state_architecture.svg</t>
+          <t>source/07_data_analytics_reporting/report_inventory.xlsx</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>svg</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>it_systems_architecture</t>
+          <t>data_analytics_reporting</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Architecture</t>
+          <t>Power BI</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>3923</v>
+        <v>19054</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>source/07_data_analytics_reporting/report_inventory.xlsx</t>
+          <t>source/07_data_analytics_reporting/dashboard_inventory.xlsx</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2366,13 +2366,13 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>19051</v>
+        <v>7783</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>source/07_data_analytics_reporting/dashboard_inventory.xlsx</t>
+          <t>source/07_data_analytics_reporting/kpi_definitions.xlsx</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2387,17 +2387,17 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Power BI</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>7776</v>
+        <v>5916</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>source/07_data_analytics_reporting/kpi_definitions.xlsx</t>
+          <t>source/07_data_analytics_reporting/data_ownership.xlsx</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2416,13 +2416,13 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>5896</v>
+        <v>5708</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>source/07_data_analytics_reporting/data_ownership.xlsx</t>
+          <t>source/07_data_analytics_reporting/data_quality_issues.xlsx</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2441,18 +2441,18 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>5691</v>
+        <v>6503</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>source/07_data_analytics_reporting/data_quality_issues.xlsx</t>
+          <t>source/07_data_analytics_reporting/lineage_map.csv</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>csv</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2466,18 +2466,18 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>6509</v>
+        <v>2611</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>source/07_data_analytics_reporting/lineage_map.csv</t>
+          <t>source/07_data_analytics_reporting/semantic_layer_assumptions.docx</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2491,18 +2491,18 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>2602</v>
+        <v>38870</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>source/07_data_analytics_reporting/semantic_layer_assumptions.docx</t>
+          <t>source/07_data_analytics_reporting/data_products.xlsx</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2516,13 +2516,13 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>38229</v>
+        <v>5647</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>source/07_data_analytics_reporting/data_products.xlsx</t>
+          <t>source/07_data_analytics_reporting/analytics_backlog.xlsx</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2541,18 +2541,18 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>5649</v>
+        <v>6177</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>source/07_data_analytics_reporting/analytics_backlog.xlsx</t>
+          <t>source/07_data_analytics_reporting/reporting_rationalization_brief.pdf</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2562,42 +2562,42 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Snowflake</t>
+          <t>Power BI</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>6188</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>source/07_data_analytics_reporting/reporting_rationalization_brief.pdf</t>
+          <t>source/08_operations_business_process/order_to_cash.docx</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>data_analytics_reporting</t>
+          <t>operations_business_process</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Power BI</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>2842</v>
+        <v>38473</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>source/08_operations_business_process/order_to_cash.docx</t>
+          <t>source/08_operations_business_process/procure_to_pay.docx</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2612,17 +2612,17 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>Coupa</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>38473</v>
+        <v>38470</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>source/08_operations_business_process/procure_to_pay.docx</t>
+          <t>source/08_operations_business_process/record_to_report.docx</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2637,17 +2637,17 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Coupa</t>
+          <t>SAP S/4HANA</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>38470</v>
+        <v>38480</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>source/08_operations_business_process/record_to_report.docx</t>
+          <t>source/08_operations_business_process/treasury_operations.docx</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2662,17 +2662,17 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>SAP S/4HANA</t>
+          <t>Kyriba TMS</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>38480</v>
+        <v>38479</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>source/08_operations_business_process/treasury_operations.docx</t>
+          <t>source/08_operations_business_process/vendor_onboarding.docx</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2687,17 +2687,17 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Kyriba TMS</t>
+          <t>Coupa</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>38479</v>
+        <v>38475</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>source/08_operations_business_process/vendor_onboarding.docx</t>
+          <t>source/08_operations_business_process/planning_cycle.docx</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2712,17 +2712,17 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Coupa</t>
+          <t>OneStream</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>38475</v>
+        <v>38474</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>source/08_operations_business_process/planning_cycle.docx</t>
+          <t>source/08_operations_business_process/management_reporting_process.docx</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2737,22 +2737,22 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>OneStream</t>
+          <t>Power BI</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>38474</v>
+        <v>38490</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>source/08_operations_business_process/management_reporting_process.docx</t>
+          <t>source/08_operations_business_process/month_end_close.pdf</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2762,22 +2762,22 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Power BI</t>
+          <t>OneStream</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>38490</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>source/08_operations_business_process/month_end_close.pdf</t>
+          <t>source/08_operations_business_process/process_kpi_baseline.xlsx</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2787,47 +2787,47 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>OneStream</t>
+          <t>ServiceNow</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>2500</v>
+        <v>5633</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>source/08_operations_business_process/process_kpi_baseline.xlsx</t>
+          <t>source/09_servicenow_support_workload/servicenow_incidents.csv</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>csv</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>operations_business_process</t>
+          <t>servicenow_support_workload</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>ServiceNow</t>
+          <t>ServiceNow ITSM</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>5631</v>
+        <v>194200</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>source/09_servicenow_support_workload/servicenow_incidents.csv</t>
+          <t>source/09_servicenow_support_workload/servicenow_events.jsonl</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>jsonl</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2841,18 +2841,18 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>194241</v>
+        <v>199163</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>source/09_servicenow_support_workload/servicenow_events.jsonl</t>
+          <t>source/09_servicenow_support_workload/enhancement_backlog.xlsx</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>jsonl</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2866,13 +2866,13 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>199104</v>
+        <v>9458</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>source/09_servicenow_support_workload/enhancement_backlog.xlsx</t>
+          <t>source/09_servicenow_support_workload/defects.xlsx</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2891,13 +2891,13 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>9450</v>
+        <v>7784</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>source/09_servicenow_support_workload/defects.xlsx</t>
+          <t>source/09_servicenow_support_workload/sla_model.xlsx</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2916,13 +2916,13 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>7785</v>
+        <v>5520</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>source/09_servicenow_support_workload/sla_model.xlsx</t>
+          <t>source/09_servicenow_support_workload/ticket_categories.xlsx</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2941,13 +2941,13 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>5519</v>
+        <v>5695</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>source/09_servicenow_support_workload/ticket_categories.xlsx</t>
+          <t>source/09_servicenow_support_workload/ticket_aging.xlsx</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2966,18 +2966,18 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>5692</v>
+        <v>5490</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>source/09_servicenow_support_workload/ticket_aging.xlsx</t>
+          <t>source/09_servicenow_support_workload/root_cause_analysis.pdf</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2991,18 +2991,18 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>5490</v>
+        <v>2729</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>source/09_servicenow_support_workload/root_cause_analysis.pdf</t>
+          <t>source/09_servicenow_support_workload/support_team_structure.xlsx</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -3016,13 +3016,13 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>2729</v>
+        <v>5610</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>source/09_servicenow_support_workload/support_team_structure.xlsx</t>
+          <t>source/09_servicenow_support_workload/automation_opportunities.xlsx</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3041,13 +3041,13 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>5607</v>
+        <v>5732</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>source/09_servicenow_support_workload/automation_opportunities.xlsx</t>
+          <t>source/10_vendors_contracts_source/si_contracts.xlsx</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3057,22 +3057,22 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>servicenow_support_workload</t>
+          <t>vendors_contracts_source</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>ServiceNow ITSM</t>
+          <t>Coupa</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>5734</v>
+        <v>6430</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>source/10_vendors_contracts_source/si_contracts.xlsx</t>
+          <t>source/10_vendors_contracts_source/software_contracts.xlsx</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3091,13 +3091,13 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>6434</v>
+        <v>6763</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>source/10_vendors_contracts_source/software_contracts.xlsx</t>
+          <t>source/10_vendors_contracts_source/bank_partner_contracts.xlsx</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3112,17 +3112,17 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Coupa</t>
+          <t>Kyriba TMS</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>6775</v>
+        <v>5881</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>source/10_vendors_contracts_source/bank_partner_contracts.xlsx</t>
+          <t>source/10_vendors_contracts_source/rate_cards.xlsx</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3137,17 +3137,17 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Kyriba TMS</t>
+          <t>Coupa</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>5877</v>
+        <v>8011</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>source/10_vendors_contracts_source/rate_cards.xlsx</t>
+          <t>source/10_vendors_contracts_source/vendor_scorecards.xlsx</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3166,13 +3166,13 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>8011</v>
+        <v>5693</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>source/10_vendors_contracts_source/vendor_scorecards.xlsx</t>
+          <t>source/10_vendors_contracts_source/sourcing_pipeline.xlsx</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -3191,13 +3191,13 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>5696</v>
+        <v>5896</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>source/10_vendors_contracts_source/sourcing_pipeline.xlsx</t>
+          <t>source/10_vendors_contracts_source/bafo_model.xlsx</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -3216,13 +3216,13 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>5889</v>
+        <v>5586</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>source/10_vendors_contracts_source/bafo_model.xlsx</t>
+          <t>source/10_vendors_contracts_source/contract_risks.xlsx</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -3241,13 +3241,13 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>5579</v>
+        <v>5912</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>source/10_vendors_contracts_source/contract_risks.xlsx</t>
+          <t>source/10_vendors_contracts_source/renewal_calendar.xlsx</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -3266,18 +3266,18 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>5909</v>
+        <v>6506</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>source/10_vendors_contracts_source/renewal_calendar.xlsx</t>
+          <t>source/10_vendors_contracts_source/rfp_requirements.docx</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -3291,18 +3291,18 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>6498</v>
+        <v>38445</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>source/10_vendors_contracts_source/rfp_requirements.docx</t>
+          <t>source/10_vendors_contracts_source/ams_contract.pdf</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3316,38 +3316,38 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>38445</v>
+        <v>2944</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>source/10_vendors_contracts_source/ams_contract.pdf</t>
+          <t>source/11_risk_controls_responsible_ai/risk_control_register.xlsx</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>vendors_contracts_source</t>
+          <t>risk_controls_responsible_ai</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Coupa</t>
+          <t>GRC</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>2944</v>
+        <v>9970</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>source/11_risk_controls_responsible_ai/risk_control_register.xlsx</t>
+          <t>source/11_risk_controls_responsible_ai/sox_controls.xlsx</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3366,13 +3366,13 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>9969</v>
+        <v>6671</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>source/11_risk_controls_responsible_ai/sox_controls.xlsx</t>
+          <t>source/11_risk_controls_responsible_ai/payment_fraud_controls.xlsx</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3387,17 +3387,17 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>GRC</t>
+          <t>Kyriba TMS</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>6669</v>
+        <v>5578</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>source/11_risk_controls_responsible_ai/payment_fraud_controls.xlsx</t>
+          <t>source/11_risk_controls_responsible_ai/segregation_of_duties.xlsx</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3412,17 +3412,17 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Kyriba TMS</t>
+          <t>SailPoint</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>5580</v>
+        <v>6087</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>source/11_risk_controls_responsible_ai/segregation_of_duties.xlsx</t>
+          <t>source/11_risk_controls_responsible_ai/audit_findings.xlsx</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3437,17 +3437,17 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>SailPoint</t>
+          <t>GRC</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>6088</v>
+        <v>6731</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>source/11_risk_controls_responsible_ai/audit_findings.xlsx</t>
+          <t>source/11_risk_controls_responsible_ai/cyber_risks.xlsx</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -3462,17 +3462,17 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>GRC</t>
+          <t>Sentinel</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>6727</v>
+        <v>5907</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>source/11_risk_controls_responsible_ai/cyber_risks.xlsx</t>
+          <t>source/11_risk_controls_responsible_ai/operational_risks.xlsx</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3487,17 +3487,17 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Sentinel</t>
+          <t>GRC</t>
         </is>
       </c>
       <c r="E114" t="n">
-        <v>5904</v>
+        <v>5790</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>source/11_risk_controls_responsible_ai/operational_risks.xlsx</t>
+          <t>source/11_risk_controls_responsible_ai/responsible_ai_controls.xlsx</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3512,17 +3512,17 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>GRC</t>
+          <t>AI Governance</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>5791</v>
+        <v>5790</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>source/11_risk_controls_responsible_ai/responsible_ai_controls.xlsx</t>
+          <t>source/11_risk_controls_responsible_ai/model_use_case_review_checklist.xlsx</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3541,18 +3541,18 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>5807</v>
+        <v>5649</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>source/11_risk_controls_responsible_ai/model_use_case_review_checklist.xlsx</t>
+          <t>source/11_risk_controls_responsible_ai/evidence_gap_register.csv</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>csv</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -3562,22 +3562,22 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>AI Governance</t>
+          <t>GRC</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>5643</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>source/11_risk_controls_responsible_ai/evidence_gap_register.csv</t>
+          <t>source/11_risk_controls_responsible_ai/ai_governance.pdf</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3587,42 +3587,42 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>GRC</t>
+          <t>AI Governance</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>1579</v>
+        <v>2914</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>source/11_risk_controls_responsible_ai/ai_governance.pdf</t>
+          <t>source/12_ai_use_cases_moves/ai_opportunity_portfolio.xlsx</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>risk_controls_responsible_ai</t>
+          <t>ai_use_cases_moves</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>AI Governance</t>
+          <t>AbarVa</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>2914</v>
+        <v>8281</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>source/12_ai_use_cases_moves/ai_opportunity_portfolio.xlsx</t>
+          <t>source/12_ai_use_cases_moves/finance_ai_use_cases.xlsx</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3641,13 +3641,13 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>8265</v>
+        <v>5990</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>source/12_ai_use_cases_moves/finance_ai_use_cases.xlsx</t>
+          <t>source/12_ai_use_cases_moves/it_modernization_use_cases.xlsx</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3666,13 +3666,13 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>5980</v>
+        <v>5968</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>source/12_ai_use_cases_moves/it_modernization_use_cases.xlsx</t>
+          <t>source/12_ai_use_cases_moves/procurement_vendor_optimization_use_cases.xlsx</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3691,13 +3691,13 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>5970</v>
+        <v>5979</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>source/12_ai_use_cases_moves/procurement_vendor_optimization_use_cases.xlsx</t>
+          <t>source/12_ai_use_cases_moves/cost_optimization_use_case.xlsx</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3716,13 +3716,13 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>6032</v>
+        <v>6012</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>source/12_ai_use_cases_moves/cost_optimization_use_case.xlsx</t>
+          <t>source/12_ai_use_cases_moves/value_realization_model.xlsx</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3741,18 +3741,18 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>6002</v>
+        <v>5993</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>source/12_ai_use_cases_moves/value_realization_model.xlsx</t>
+          <t>source/12_ai_use_cases_moves/treasury_kyriba_success_use_case.pdf</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3762,22 +3762,22 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>AbarVa</t>
+          <t>Kyriba TMS</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>5978</v>
+        <v>2595</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>source/12_ai_use_cases_moves/treasury_kyriba_success_use_case.pdf</t>
+          <t>source/12_ai_use_cases_moves/reporting_rationalization_use_case.docx</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>docx</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3787,17 +3787,17 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Kyriba TMS</t>
+          <t>Power BI</t>
         </is>
       </c>
       <c r="E126" t="n">
-        <v>2595</v>
+        <v>38291</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>source/12_ai_use_cases_moves/reporting_rationalization_use_case.docx</t>
+          <t>source/12_ai_use_cases_moves/human_agent_operating_model.docx</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3812,22 +3812,22 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Power BI</t>
+          <t>AbarVa</t>
         </is>
       </c>
       <c r="E127" t="n">
-        <v>38291</v>
+        <v>38464</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>source/12_ai_use_cases_moves/human_agent_operating_model.docx</t>
+          <t>source/12_ai_use_cases_moves/ai_moves_portfolio_summary.md</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>md</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3841,32 +3841,182 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>38464</v>
+        <v>836</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>source/12_ai_use_cases_moves/ai_moves_portfolio_summary.md</t>
+          <t>source/06_it_systems_architecture/current_state_architecture.svg</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>svg</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
+          <t>it_systems_architecture</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>20866</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>source/06_it_systems_architecture/integration_architecture_diagram.svg</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>it_systems_architecture</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>SAP PI/PO</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>15029</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>source/05_treasury_kyriba/kyriba_connectivity_architecture.svg</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>treasury_kyriba</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Kyriba TMS</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>14149</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>source/07_data_analytics_reporting/data_platform_architecture.svg</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>data_analytics_reporting</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Snowflake</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>12413</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>source/11_risk_controls_responsible_ai/security_zero_trust_architecture.svg</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>risk_controls_responsible_ai</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Microsoft Sentinel</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>9924</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>source/12_ai_use_cases_moves/ai_agent_reference_architecture.svg</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
           <t>ai_use_cases_moves</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr">
+      <c r="D134" t="inlineStr">
         <is>
           <t>AbarVa</t>
         </is>
       </c>
-      <c r="E129" t="n">
-        <v>836</v>
+      <c r="E134" t="n">
+        <v>11866</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>source/03_strategy_initiatives/roadmap_2026_2027.svg</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>strategy_initiatives</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>6563</v>
       </c>
     </row>
   </sheetData>

</xml_diff>